<commit_message>
Updated the DR by SNR files
</commit_message>
<xml_diff>
--- a/data/dynamic_test/dynamic_test.xlsx
+++ b/data/dynamic_test/dynamic_test.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jon/usra2026/data/dynamic_test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99C3470D-D2F8-5E46-A20D-1C4C81097BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70309A46-20BC-C549-8F72-AA4F0B1A93FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12100" yWindow="500" windowWidth="16700" windowHeight="17500" activeTab="1" xr2:uid="{242F5C09-2629-5B4F-9A1A-8A58ACE0AAAB}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="1" xr2:uid="{242F5C09-2629-5B4F-9A1A-8A58ACE0AAAB}"/>
   </bookViews>
   <sheets>
     <sheet name="dynamic_test_3hop" sheetId="1" r:id="rId1"/>
@@ -135,7 +135,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="209">
   <si>
     <t>localID</t>
   </si>
@@ -756,6 +756,12 @@
   </si>
   <si>
     <t>closest node</t>
+  </si>
+  <si>
+    <t>SNR (normalized)</t>
+  </si>
+  <si>
+    <t>distance to closest node relative to SNR</t>
   </si>
 </sst>
 </file>
@@ -7420,16 +7426,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EDD6C84-90E4-EC4A-821B-D1BE88657BA9}">
-  <dimension ref="A1:W63"/>
+  <dimension ref="A1:Y63"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="15" max="15" width="15.33203125" customWidth="1"/>
     <col min="17" max="17" width="29.5" customWidth="1"/>
     <col min="18" max="18" width="19.6640625" customWidth="1"/>
     <col min="20" max="20" width="12.1640625" customWidth="1"/>
+    <col min="24" max="24" width="17.1640625" customWidth="1"/>
+    <col min="25" max="25" width="36.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:25" s="2" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -7499,8 +7507,14 @@
       <c r="W1" s="2" t="s">
         <v>206</v>
       </c>
+      <c r="X1" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>208</v>
+      </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7617,8 +7631,16 @@
         <f>MIN(Q2:V2)</f>
         <v>23.001235656757817</v>
       </c>
+      <c r="X2">
+        <f>H2+15</f>
+        <v>24.5</v>
+      </c>
+      <c r="Y2">
+        <f>W2/X2</f>
+        <v>0.93882594517378848</v>
+      </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7727,8 +7749,16 @@
         <f t="shared" ref="W3:W63" si="2">MIN(Q3:V3)</f>
         <v>23.001235656757817</v>
       </c>
+      <c r="X3">
+        <f t="shared" ref="X3:X63" si="3">H3+15</f>
+        <v>24.25</v>
+      </c>
+      <c r="Y3">
+        <f t="shared" ref="Y3:Y63" si="4">W3/X3</f>
+        <v>0.94850456316527076</v>
+      </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7837,8 +7867,16 @@
         <f t="shared" si="2"/>
         <v>23.001235656757817</v>
       </c>
+      <c r="X4">
+        <f t="shared" si="3"/>
+        <v>25.5</v>
+      </c>
+      <c r="Y4">
+        <f t="shared" si="4"/>
+        <v>0.90200924144148298</v>
+      </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7947,8 +7985,16 @@
         <f t="shared" si="2"/>
         <v>23.001235656757817</v>
       </c>
+      <c r="X5">
+        <f t="shared" si="3"/>
+        <v>25.5</v>
+      </c>
+      <c r="Y5">
+        <f t="shared" si="4"/>
+        <v>0.90200924144148298</v>
+      </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
@@ -8057,8 +8103,16 @@
         <f t="shared" si="2"/>
         <v>23.001235656757817</v>
       </c>
+      <c r="X6">
+        <f t="shared" si="3"/>
+        <v>25.25</v>
+      </c>
+      <c r="Y6">
+        <f t="shared" si="4"/>
+        <v>0.91094002601021062</v>
+      </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8167,8 +8221,16 @@
         <f t="shared" si="2"/>
         <v>23.027757495974619</v>
       </c>
+      <c r="X7">
+        <f t="shared" si="3"/>
+        <v>24.25</v>
+      </c>
+      <c r="Y7">
+        <f t="shared" si="4"/>
+        <v>0.94959824725668529</v>
+      </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8277,8 +8339,16 @@
         <f t="shared" si="2"/>
         <v>23.027757495974619</v>
       </c>
+      <c r="X8">
+        <f t="shared" si="3"/>
+        <v>25.25</v>
+      </c>
+      <c r="Y8">
+        <f t="shared" si="4"/>
+        <v>0.91199039588018294</v>
+      </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8387,8 +8457,16 @@
         <f t="shared" si="2"/>
         <v>23.027757495974619</v>
       </c>
+      <c r="X9">
+        <f t="shared" si="3"/>
+        <v>24.5</v>
+      </c>
+      <c r="Y9">
+        <f t="shared" si="4"/>
+        <v>0.93990846922345384</v>
+      </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>9</v>
       </c>
@@ -8497,8 +8575,16 @@
         <f t="shared" si="2"/>
         <v>23.132489276433567</v>
       </c>
+      <c r="X10">
+        <f t="shared" si="3"/>
+        <v>24.5</v>
+      </c>
+      <c r="Y10">
+        <f t="shared" si="4"/>
+        <v>0.94418323577279861</v>
+      </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>10</v>
       </c>
@@ -8607,8 +8693,16 @@
         <f t="shared" si="2"/>
         <v>23.132489276433567</v>
       </c>
+      <c r="X11">
+        <f t="shared" si="3"/>
+        <v>25</v>
+      </c>
+      <c r="Y11">
+        <f t="shared" si="4"/>
+        <v>0.92529957105734273</v>
+      </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>11</v>
       </c>
@@ -8717,8 +8811,16 @@
         <f t="shared" si="2"/>
         <v>23.132489276433567</v>
       </c>
+      <c r="X12">
+        <f t="shared" si="3"/>
+        <v>24.75</v>
+      </c>
+      <c r="Y12">
+        <f t="shared" si="4"/>
+        <v>0.93464603137105318</v>
+      </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>12</v>
       </c>
@@ -8827,8 +8929,16 @@
         <f t="shared" si="2"/>
         <v>12.972932659475628</v>
       </c>
+      <c r="X13">
+        <f t="shared" si="3"/>
+        <v>24.25</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="4"/>
+        <v>0.53496629523610839</v>
+      </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>13</v>
       </c>
@@ -8937,8 +9047,16 @@
         <f t="shared" si="2"/>
         <v>18.070645466124741</v>
       </c>
+      <c r="X14">
+        <f t="shared" si="3"/>
+        <v>23.75</v>
+      </c>
+      <c r="Y14">
+        <f t="shared" si="4"/>
+        <v>0.76086928278419963</v>
+      </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>15</v>
       </c>
@@ -9047,8 +9165,16 @@
         <f t="shared" si="2"/>
         <v>54.62703002768037</v>
       </c>
+      <c r="X15">
+        <f t="shared" si="3"/>
+        <v>24.25</v>
+      </c>
+      <c r="Y15">
+        <f t="shared" si="4"/>
+        <v>2.2526610320692937</v>
+      </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>19</v>
       </c>
@@ -9157,8 +9283,16 @@
         <f t="shared" si="2"/>
         <v>158.01266200674121</v>
       </c>
+      <c r="X16">
+        <f t="shared" si="3"/>
+        <v>21.75</v>
+      </c>
+      <c r="Y16">
+        <f t="shared" si="4"/>
+        <v>7.264949977321435</v>
+      </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>20</v>
       </c>
@@ -9267,8 +9401,16 @@
         <f t="shared" si="2"/>
         <v>152.68317332984668</v>
       </c>
+      <c r="X17">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y17">
+        <f t="shared" si="4"/>
+        <v>6.567018207735341</v>
+      </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>21</v>
       </c>
@@ -9377,8 +9519,16 @@
         <f t="shared" si="2"/>
         <v>145.18579859693344</v>
       </c>
+      <c r="X18">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y18">
+        <f t="shared" si="4"/>
+        <v>6.2445504772874596</v>
+      </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>23</v>
       </c>
@@ -9487,8 +9637,16 @@
         <f t="shared" si="2"/>
         <v>86.401392629313662</v>
       </c>
+      <c r="X19">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y19">
+        <f t="shared" si="4"/>
+        <v>3.7565822882310287</v>
+      </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>24</v>
       </c>
@@ -9597,8 +9755,16 @@
         <f t="shared" si="2"/>
         <v>61.038947737575356</v>
       </c>
+      <c r="X20">
+        <f t="shared" si="3"/>
+        <v>22.25</v>
+      </c>
+      <c r="Y20">
+        <f t="shared" si="4"/>
+        <v>2.7433234938236115</v>
+      </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>25</v>
       </c>
@@ -9707,8 +9873,16 @@
         <f t="shared" si="2"/>
         <v>32.08852351764088</v>
       </c>
+      <c r="X21">
+        <f t="shared" si="3"/>
+        <v>22.75</v>
+      </c>
+      <c r="Y21">
+        <f t="shared" si="4"/>
+        <v>1.4104845502259726</v>
+      </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>26</v>
       </c>
@@ -9817,8 +9991,16 @@
         <f t="shared" si="2"/>
         <v>51.894291674235411</v>
       </c>
+      <c r="X22">
+        <f t="shared" si="3"/>
+        <v>4.75</v>
+      </c>
+      <c r="Y22">
+        <f t="shared" si="4"/>
+        <v>10.925114036681139</v>
+      </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>28</v>
       </c>
@@ -9927,8 +10109,16 @@
         <f t="shared" si="2"/>
         <v>104.57694191588507</v>
       </c>
+      <c r="X23">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y23">
+        <f t="shared" si="4"/>
+        <v>4.5468235615602204</v>
+      </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>29</v>
       </c>
@@ -10037,8 +10227,16 @@
         <f t="shared" si="2"/>
         <v>110.70306274462978</v>
       </c>
+      <c r="X24">
+        <f t="shared" si="3"/>
+        <v>22.75</v>
+      </c>
+      <c r="Y24">
+        <f t="shared" si="4"/>
+        <v>4.8660686920716385</v>
+      </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>31</v>
       </c>
@@ -10147,8 +10345,16 @@
         <f t="shared" si="2"/>
         <v>152.72629118229182</v>
       </c>
+      <c r="X25">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y25">
+        <f t="shared" si="4"/>
+        <v>6.6402735296648618</v>
+      </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>32</v>
       </c>
@@ -10257,8 +10463,16 @@
         <f t="shared" si="2"/>
         <v>184.75073430159932</v>
       </c>
+      <c r="X26">
+        <f t="shared" si="3"/>
+        <v>21.5</v>
+      </c>
+      <c r="Y26">
+        <f t="shared" si="4"/>
+        <v>8.593057409376712</v>
+      </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>33</v>
       </c>
@@ -10367,8 +10581,16 @@
         <f t="shared" si="2"/>
         <v>209.08714750394273</v>
       </c>
+      <c r="X27">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y27">
+        <f t="shared" si="4"/>
+        <v>8.9929955915674284</v>
+      </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>35</v>
       </c>
@@ -10477,8 +10699,16 @@
         <f t="shared" si="2"/>
         <v>147.22384101311403</v>
       </c>
+      <c r="X28">
+        <f t="shared" si="3"/>
+        <v>22.75</v>
+      </c>
+      <c r="Y28">
+        <f t="shared" si="4"/>
+        <v>6.4713776269500674</v>
+      </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>36</v>
       </c>
@@ -10587,8 +10817,16 @@
         <f t="shared" si="2"/>
         <v>115.38010019988579</v>
       </c>
+      <c r="X29">
+        <f t="shared" si="3"/>
+        <v>22.5</v>
+      </c>
+      <c r="Y29">
+        <f t="shared" si="4"/>
+        <v>5.1280044533282574</v>
+      </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>38</v>
       </c>
@@ -10697,8 +10935,16 @@
         <f t="shared" si="2"/>
         <v>110.1859575583656</v>
       </c>
+      <c r="X30">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y30">
+        <f t="shared" si="4"/>
+        <v>4.739180970252284</v>
+      </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>39</v>
       </c>
@@ -10807,8 +11053,16 @@
         <f t="shared" si="2"/>
         <v>113.68520610296713</v>
       </c>
+      <c r="X31">
+        <f t="shared" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="Y31">
+        <f t="shared" si="4"/>
+        <v>4.7368835876236304</v>
+      </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>40</v>
       </c>
@@ -10917,8 +11171,16 @@
         <f t="shared" si="2"/>
         <v>116.21684031128693</v>
       </c>
+      <c r="X32">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y32">
+        <f t="shared" si="4"/>
+        <v>5.0529061004907359</v>
+      </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>42</v>
       </c>
@@ -11027,8 +11289,16 @@
         <f t="shared" si="2"/>
         <v>101.12117471567765</v>
       </c>
+      <c r="X33">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y33">
+        <f t="shared" si="4"/>
+        <v>4.3492978372334479</v>
+      </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>45</v>
       </c>
@@ -11137,8 +11407,16 @@
         <f t="shared" si="2"/>
         <v>90.950799847059073</v>
       </c>
+      <c r="X34">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y34">
+        <f t="shared" si="4"/>
+        <v>3.9543826020460466</v>
+      </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>46</v>
       </c>
@@ -11247,8 +11525,16 @@
         <f t="shared" si="2"/>
         <v>88.043327244252765</v>
       </c>
+      <c r="X35">
+        <f t="shared" si="3"/>
+        <v>24.75</v>
+      </c>
+      <c r="Y35">
+        <f t="shared" si="4"/>
+        <v>3.55730615128294</v>
+      </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>51</v>
       </c>
@@ -11357,8 +11643,16 @@
         <f t="shared" si="2"/>
         <v>88.081801444626493</v>
       </c>
+      <c r="X36">
+        <f t="shared" si="3"/>
+        <v>24.25</v>
+      </c>
+      <c r="Y36">
+        <f t="shared" si="4"/>
+        <v>3.6322392348299584</v>
+      </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>53</v>
       </c>
@@ -11467,8 +11761,16 @@
         <f t="shared" si="2"/>
         <v>39.600653963968725</v>
       </c>
+      <c r="X37">
+        <f t="shared" si="3"/>
+        <v>22.75</v>
+      </c>
+      <c r="Y37">
+        <f t="shared" si="4"/>
+        <v>1.7406880863282956</v>
+      </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>54</v>
       </c>
@@ -11577,8 +11879,16 @@
         <f t="shared" si="2"/>
         <v>40.866841727460546</v>
       </c>
+      <c r="X38">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y38">
+        <f t="shared" si="4"/>
+        <v>1.7768192055417629</v>
+      </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>55</v>
       </c>
@@ -11687,8 +11997,16 @@
         <f t="shared" si="2"/>
         <v>43.420763783365146</v>
       </c>
+      <c r="X39">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y39">
+        <f t="shared" si="4"/>
+        <v>1.8675597326178557</v>
+      </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>56</v>
       </c>
@@ -11797,8 +12115,16 @@
         <f t="shared" si="2"/>
         <v>44.770175206834999</v>
       </c>
+      <c r="X40">
+        <f t="shared" si="3"/>
+        <v>22.25</v>
+      </c>
+      <c r="Y40">
+        <f t="shared" si="4"/>
+        <v>2.0121427059251684</v>
+      </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>57</v>
       </c>
@@ -11907,8 +12233,16 @@
         <f t="shared" si="2"/>
         <v>37.541671163667587</v>
       </c>
+      <c r="X41">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y41">
+        <f t="shared" si="4"/>
+        <v>1.6146955339211866</v>
+      </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>58</v>
       </c>
@@ -12017,8 +12351,16 @@
         <f t="shared" si="2"/>
         <v>31.71871767051956</v>
       </c>
+      <c r="X42">
+        <f t="shared" si="3"/>
+        <v>22.75</v>
+      </c>
+      <c r="Y42">
+        <f t="shared" si="4"/>
+        <v>1.3942293481547059</v>
+      </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>59</v>
       </c>
@@ -12127,8 +12469,16 @@
         <f t="shared" si="2"/>
         <v>51.105475940217701</v>
       </c>
+      <c r="X43">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y43">
+        <f t="shared" si="4"/>
+        <v>2.2219772147920738</v>
+      </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>60</v>
       </c>
@@ -12237,8 +12587,16 @@
         <f t="shared" si="2"/>
         <v>82.083853785764163</v>
       </c>
+      <c r="X44">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y44">
+        <f t="shared" si="4"/>
+        <v>3.5304883348715768</v>
+      </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>61</v>
       </c>
@@ -12347,8 +12705,16 @@
         <f t="shared" si="2"/>
         <v>115.03435287833788</v>
       </c>
+      <c r="X45">
+        <f t="shared" si="3"/>
+        <v>23.75</v>
+      </c>
+      <c r="Y45">
+        <f t="shared" si="4"/>
+        <v>4.8435517001405426</v>
+      </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>62</v>
       </c>
@@ -12457,8 +12823,16 @@
         <f t="shared" si="2"/>
         <v>107.47646793317809</v>
       </c>
+      <c r="X46">
+        <f t="shared" si="3"/>
+        <v>23.75</v>
+      </c>
+      <c r="Y46">
+        <f t="shared" si="4"/>
+        <v>4.5253249656074983</v>
+      </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>63</v>
       </c>
@@ -12567,8 +12941,16 @@
         <f t="shared" si="2"/>
         <v>85.921823094855966</v>
       </c>
+      <c r="X47">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y47">
+        <f t="shared" si="4"/>
+        <v>3.6955622836497191</v>
+      </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>64</v>
       </c>
@@ -12677,8 +13059,16 @@
         <f t="shared" si="2"/>
         <v>71.430806392474395</v>
       </c>
+      <c r="X48">
+        <f t="shared" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="Y48">
+        <f t="shared" si="4"/>
+        <v>2.976283599686433</v>
+      </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>66</v>
       </c>
@@ -12787,8 +13177,16 @@
         <f t="shared" si="2"/>
         <v>124.11873512850565</v>
       </c>
+      <c r="X49">
+        <f t="shared" si="3"/>
+        <v>23.25</v>
+      </c>
+      <c r="Y49">
+        <f t="shared" si="4"/>
+        <v>5.3384402205808881</v>
+      </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>68</v>
       </c>
@@ -12897,8 +13295,16 @@
         <f t="shared" si="2"/>
         <v>169.23897766774414</v>
       </c>
+      <c r="X50">
+        <f t="shared" si="3"/>
+        <v>22.5</v>
+      </c>
+      <c r="Y50">
+        <f t="shared" si="4"/>
+        <v>7.5217323407886285</v>
+      </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>70</v>
       </c>
@@ -13007,8 +13413,16 @@
         <f t="shared" si="2"/>
         <v>191.7792615434185</v>
       </c>
+      <c r="X51">
+        <f t="shared" si="3"/>
+        <v>24.75</v>
+      </c>
+      <c r="Y51">
+        <f t="shared" si="4"/>
+        <v>7.7486570320573129</v>
+      </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>71</v>
       </c>
@@ -13117,8 +13531,16 @@
         <f t="shared" si="2"/>
         <v>144.2345308137551</v>
       </c>
+      <c r="X52">
+        <f t="shared" si="3"/>
+        <v>24.75</v>
+      </c>
+      <c r="Y52">
+        <f t="shared" si="4"/>
+        <v>5.8276578106567714</v>
+      </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>73</v>
       </c>
@@ -13227,8 +13649,16 @@
         <f t="shared" si="2"/>
         <v>106.56082770247741</v>
       </c>
+      <c r="X53">
+        <f t="shared" si="3"/>
+        <v>22.25</v>
+      </c>
+      <c r="Y53">
+        <f t="shared" si="4"/>
+        <v>4.7892506832574115</v>
+      </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>74</v>
       </c>
@@ -13337,8 +13767,16 @@
         <f t="shared" si="2"/>
         <v>93.321276072509093</v>
       </c>
+      <c r="X54">
+        <f t="shared" si="3"/>
+        <v>23.5</v>
+      </c>
+      <c r="Y54">
+        <f t="shared" si="4"/>
+        <v>3.9711181307450678</v>
+      </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>75</v>
       </c>
@@ -13447,8 +13885,16 @@
         <f t="shared" si="2"/>
         <v>89.145446246405541</v>
       </c>
+      <c r="X55">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y55">
+        <f t="shared" si="4"/>
+        <v>3.8758889672350234</v>
+      </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>77</v>
       </c>
@@ -13557,8 +14003,16 @@
         <f t="shared" si="2"/>
         <v>46.457496228992845</v>
       </c>
+      <c r="X56">
+        <f t="shared" si="3"/>
+        <v>11.25</v>
+      </c>
+      <c r="Y56">
+        <f t="shared" si="4"/>
+        <v>4.12955522035492</v>
+      </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>78</v>
       </c>
@@ -13667,8 +14121,16 @@
         <f t="shared" si="2"/>
         <v>51.099978733045027</v>
       </c>
+      <c r="X57">
+        <f t="shared" si="3"/>
+        <v>14.75</v>
+      </c>
+      <c r="Y57">
+        <f t="shared" si="4"/>
+        <v>3.4644053378335613</v>
+      </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>79</v>
       </c>
@@ -13777,8 +14239,16 @@
         <f t="shared" si="2"/>
         <v>47.498363340718278</v>
       </c>
+      <c r="X58">
+        <f t="shared" si="3"/>
+        <v>19.75</v>
+      </c>
+      <c r="Y58">
+        <f t="shared" si="4"/>
+        <v>2.4049804223148494</v>
+      </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>80</v>
       </c>
@@ -13887,8 +14357,16 @@
         <f t="shared" si="2"/>
         <v>16.656219071636333</v>
       </c>
+      <c r="X59">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y59">
+        <f t="shared" si="4"/>
+        <v>0.72418343789723183</v>
+      </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>81</v>
       </c>
@@ -13997,8 +14475,16 @@
         <f t="shared" si="2"/>
         <v>21.795116976853119</v>
       </c>
+      <c r="X60">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="Y60">
+        <f t="shared" si="4"/>
+        <v>0.94761378160230958</v>
+      </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>82</v>
       </c>
@@ -14107,8 +14593,16 @@
         <f t="shared" si="2"/>
         <v>21.401170961053595</v>
       </c>
+      <c r="X61">
+        <f t="shared" si="3"/>
+        <v>24</v>
+      </c>
+      <c r="Y61">
+        <f t="shared" si="4"/>
+        <v>0.8917154567105664</v>
+      </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>83</v>
       </c>
@@ -14217,8 +14711,16 @@
         <f t="shared" si="2"/>
         <v>19.975623676386199</v>
       </c>
+      <c r="X62">
+        <f t="shared" si="3"/>
+        <v>25.5</v>
+      </c>
+      <c r="Y62">
+        <f t="shared" si="4"/>
+        <v>0.78335779123083138</v>
+      </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>84</v>
       </c>
@@ -14326,6 +14828,14 @@
       <c r="W63">
         <f t="shared" si="2"/>
         <v>33.062823279114916</v>
+      </c>
+      <c r="X63">
+        <f t="shared" si="3"/>
+        <v>24.5</v>
+      </c>
+      <c r="Y63">
+        <f t="shared" si="4"/>
+        <v>1.3495029909842824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>